<commit_message>
Task sheet: module column, deadline order, reassigned owners; add TASK_BRIEFS.md
</commit_message>
<xml_diff>
--- a/planning/tasks_week_2026-09-28.xlsx
+++ b/planning/tasks_week_2026-09-28.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tasks'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tasks'!$A$1:$I$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36,7 +36,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +46,41 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DAEEF3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2DCDB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -69,8 +104,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -463,17 +519,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -484,35 +541,40 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Depends on</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -521,938 +583,1053 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>T01</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Label CS workbook</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>annotator_4_CS_majors.xlsx — 413 rows (60 overlap + 293 training + 60 test)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Team</t>
+          <t>Entrepreneurial data</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Decide target dataset sizes</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>How many seed + test items the entrepreneurial set needs</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sat 03 Oct</t>
+          <t>Lumia</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Overlap 60 must be labelled independently, no discussion, or kappa is void</t>
+          <t>Tue 29 Sep</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>~100 non-distorted for +/-10% specificity CI; ~20/class -&gt; 200-300 for per-class</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>T02</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Label psych workbooks</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>annotator_1 Laiba 421 / annotator_2 Reesha 418 / annotator_3 Hurema 415 rows</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Laiba</t>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Transfer evaluation</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>CBT-Bench: acquire + map labels + run on org dataset finetuned model</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Psychotherapy-LLM/CBT-Bench on HuggingFace; CBT-CD split, 146 items, 10 classes</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Sat 03 Oct</t>
+          <t>Izza</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>~5h 10m each at 45 s/row; unfinished rows are acceptable</t>
+          <t>Wed 30 Sep</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Write an explicit label mapping; record how many items had to be dropped</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>T03</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Merge labels + agreement</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Run scripts/relabel_agreement.py on returned workbooks</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Nayab</t>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Span selection</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Span approach: literature + decision</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>BIO token tagging vs sentence classification vs extractive QA</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sun 04 Oct</t>
+          <t>Lumia</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Wed 30 Sep</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>T01, T02</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Produces merged_labels.csv, agreement_report.md, unsure_for_adjudication.csv</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Recommendation: sentence-level — annotators flagged sentences, report promises it</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>T04</t>
+          <t>T17</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Adjudicate Unsure rows</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Psych annotators resolve rows flagged Unsure</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Laiba</t>
+          <t>Entrepreneurial data</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Scraping: sources + ToS check</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Pick sources, confirm terms of service and redistribution limits</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Tue 06 Oct</t>
+          <t>Izza</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Wed 30 Sep</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>T03</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Nobody owned this before; needed before the labels are final</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Scraped text can be republished only as derived data in most cases</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T05</t>
+          <t>T19</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Separate errors from redefinitions</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Split label changes into genuine errors vs calibrated-pessimism redefinition</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Nayab</t>
+          <t>Entrepreneurial data</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Circulate form + start thread</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Post to relevant entrepreneurial groups/sites; collect responses</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Tue 06 Oct</t>
+          <t>Lumia</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Wed 30 Sep</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>T03</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Original annotation had no justified-concern rule; keep the two countable apart</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Consent + anonymisation first. Responses are EVALUATION ONLY, never prompts</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T06</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Back-translation augmentation</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Inflate under-represented classes in the relabelled train split</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Span selection</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Build sentence labels from spans</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Split into sentences; label the one containing the gold span; use find_span offsets</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Lumia</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Thu 08 Oct</t>
-        </is>
-      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Fri 02 Oct</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>T03, T04</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>TRAIN ONLY. Augmented rows stay in their source row's split or it is leakage</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Current span_crop/span_marked modes are ORACLE; the selector does not exist yet</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>T07</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Decide span handling for augmented rows</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Back-translation breaks 'Distorted part' offsets</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Lumia</t>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Model tuning</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Hyperparameter tuning</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>LR (2e-5/3e-5/5e-5), epochs, max_length, weight decay on the original dataset</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Wed 07 Oct</t>
+          <t>Izza</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Fri 02 Oct</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>T06</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Either re-translate + re-locate the span, or mark rows classification-only</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Val only. Confirm the winner across all 3 seeds; single-seed wins are noise</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>T08</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Hand-check augmented samples</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>30 rows per augmented class: did the distortion cue survive?</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Model tuning</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Over/underfitting diagnosis</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Train vs val loss curves per epoch; early stop on val macro-F1</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Izza</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Fri 09 Oct</t>
-        </is>
-      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Fri 02 Oct</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>T06</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>'I'll never get funding' -&gt; 'I might not' is no longer fortune-telling</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>~2,000 train rows: expect overfitting from epoch 3-4</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>T09</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>CBT-Bench: acquire + map labels</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Psychotherapy-LLM/CBT-Bench on HuggingFace; CBT-CD split, 146 items, 10 classes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Izza</t>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Re-annotation</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Label CS workbook</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>annotator_4_CS_majors.xlsx — 413 rows (60 overlap + 293 training + 60 test)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Wed 30 Sep</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Write an explicit label mapping; record how many items had to be dropped</t>
+          <t>Sat 03 Oct</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Overlap 60 must be labelled independently, no discussion, or kappa is void</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>T10</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Evaluate fine-tuned model on CBT-Bench</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Transfer test of the TherapistQA-trained model</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Izza</t>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Re-annotation</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Label psych workbooks</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>annotator_1 Laiba 421 / annotator_2 Reesha 418 / annotator_3 Hurema 415 rows</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Fri 02 Oct</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Sat 03 Oct</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>T09</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Only 146 items (~15/class): report support counts, no headline single number</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>~5h 10m each at 45 s/row; unfinished rows are acceptable</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>T11</t>
+          <t>T18</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Span approach: literature + decision</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>BIO token tagging vs sentence classification vs extractive QA</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Nayab</t>
+          <t>Entrepreneurial data</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Scrape entrepreneurial text</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Volume set by T16; cleaning and de-duplication included</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Wed 30 Sep</t>
+          <t>Izza</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Recommendation: sentence-level — annotators flagged sentences, report promises it</t>
+          <t>Sat 03 Oct</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Unlabelled at this stage; labels come later with Laiba</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>T12</t>
+          <t>T20</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Build sentence labels from spans</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Split into sentences; label the one containing the gold span; use find_span offsets</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Nayab</t>
+          <t>Entrepreneurial data</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Triage form responses</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Keep responses usable for the entrepreneurial set</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Fri 02 Oct</t>
+          <t>Lumia</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Sat 03 Oct</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>T11</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Current span_crop/span_marked modes are ORACLE; the selector does not exist yet</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>T19</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Held out at natural class distribution; do not balance</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>T13</t>
+          <t>T21</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Train + evaluate span selector</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Sentence accuracy and span overlap, reported separately from classification</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Nayab</t>
+          <t>Entrepreneurial data</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Compile entrepreneurial dataset (unlabelled)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Merge scraped + form text into one schema, ready for labelling</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Thu 08 Oct</t>
+          <t>Team</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Sat 03 Oct</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>T12</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Report the 0.402 oracle as an upper bound and the selector's cost as the gap</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>T18, T20</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>WEEK GOAL. Labels follow later with Laiba and the team</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>T14</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Hyperparameter tuning</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>LR (2e-5/3e-5/5e-5), epochs, max_length, weight decay on the original dataset</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Re-annotation</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Merge labels + agreement</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Run scripts/relabel_agreement.py on returned workbooks</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Lumia</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Fri 02 Oct</t>
-        </is>
-      </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Val only. Confirm the winner across all 3 seeds; single-seed wins are noise</t>
+          <t>Sun 04 Oct</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>T01, T02</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Produces merged_labels.csv, agreement_report.md, unsure_for_adjudication.csv</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>T15</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Over/underfitting diagnosis</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Train vs val loss curves per epoch; early stop on val macro-F1</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Lumia</t>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Specificity set</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Seed the justified-concern set</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Harvest calibrated-pessimism rows from the relabelling output</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Fri 02 Oct</t>
+          <t>Nayab</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Mon 05 Oct</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>T14</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>~2,000 train rows: expect overfitting from epoch 3-4</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Real, human-verified justified concerns; clinical topic, entrepreneurial rewrite needed</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>T16</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Decide target dataset sizes</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>How many seed + test items the entrepreneurial set needs</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Nayab</t>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Re-annotation</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Adjudicate Unsure rows</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Psych annotators resolve rows flagged Unsure</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Tue 29 Sep</t>
+          <t>Izza</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>~100 non-distorted for +/-10% specificity CI; ~20/class -&gt; 200-300 for per-class</t>
+          <t>Tue 06 Oct</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Needed before the labels are final</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>T17</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Scraping: sources + ToS check</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Pick sources, confirm terms of service and redistribution limits</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Izza</t>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Re-annotation</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Separate errors from redefinitions</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Split label changes into genuine errors vs calibrated-pessimism redefinition</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Wed 30 Sep</t>
+          <t>Lumia</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Tue 06 Oct</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>T16</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Scraped text can be republished only as derived data in most cases</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Original annotation had no justified-concern rule; keep the two countable apart</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>T18</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Scrape entrepreneurial text</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Volume set by T16; cleaning and de-duplication included</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Izza</t>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Data augmentation</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Decide span handling for augmented rows</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Back-translation breaks 'Distorted part' offsets</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Sat 03 Oct</t>
+          <t>Lumia</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Wed 07 Oct</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>T17</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Unlabelled at this stage; labels come later with Laiba</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>MOVED BEFORE T06: it is a design decision augmentation depends on, not a follow-up</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>T19</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Circulate form + start thread</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Post to relevant entrepreneurial groups/sites; collect responses</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+          <t>T06</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Data augmentation</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Back-translation augmentation</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Inflate under-represented classes in the relabelled train split</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Lumia</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Wed 30 Sep</t>
-        </is>
-      </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Consent + anonymisation first. Responses are EVALUATION ONLY, never prompts</t>
+          <t>Thu 08 Oct</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>T03, T04, T07</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>TRAIN ONLY. Augmented rows stay in their source row's split or it is leakage</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>T20</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Triage form responses</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Keep responses usable for the entrepreneurial set</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Span selection</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Train + evaluate span selector</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Sentence accuracy and span overlap, reported separately from classification</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Lumia</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Sat 03 Oct</t>
-        </is>
-      </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Thu 08 Oct</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>T19</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Held out at natural class distribution; do not balance</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Report the 0.402 oracle as an upper bound and the selector's cost as the gap</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>T21</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Compile entrepreneurial dataset (unlabelled)</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Merge scraped + form text into one schema, ready for labelling</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Team</t>
+          <t>T08</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Data augmentation</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Hand-check augmented samples</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>30 rows per augmented class: did the distortion cue survive?</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Sat 03 Oct</t>
+          <t>Izza</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Fri 09 Oct</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>T18, T20</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>WEEK GOAL. Labels follow later with Laiba and the team</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>T06</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>'I'll never get funding' -&gt; 'I might not' is no longer fortune-telling</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Specificity set</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Write challenge-set pairs</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>20 matched justified/distorted pairs per distortion family</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Fri 09 Oct</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
           <t>T22</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Seed the justified-concern set</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Harvest calibrated-pessimism rows from the relabelling output</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Nayab</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Mon 05 Oct</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>T03</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Real, human-verified justified concerns; clinical topic, entrepreneurial rewrite needed</t>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Matched pairs give controls for free and block style shortcuts</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>T23</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Write challenge-set pairs</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>20 matched justified/distorted pairs per distortion family</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Team</t>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Transfer evaluation</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Evaluate fine-tuned model with relabelled+augmented dataset on CBT-Bench</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Transfer test of the relabelled + augmented model</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Fri 09 Oct</t>
+          <t>Izza</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Sat 10 Oct</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>T22</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Matched pairs give controls for free and block style shortcuts</t>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>T06, T08, T09</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>DATE MOVED from Fri 02 Oct: it needs the augmented data, which lands Thu 08 Oct</t>
         </is>
       </c>
     </row>
@@ -1462,60 +1639,65 @@
           <t>T24</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Specificity set</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Style-leak check on challenge set</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>TF-IDF + logistic regression must score near chance on justified vs distorted</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Nayab</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Sat 10 Oct</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
           <t>T23</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>If it separates them easily (&gt;0.75 F1) the set leaks surface cues — rewrite</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H25"/>
-  <conditionalFormatting sqref="A2:H25">
+  <autoFilter ref="A1:I25"/>
+  <conditionalFormatting sqref="A2:I25">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
-      <formula>$F2="In progress"</formula>
+      <formula>$G2="In progress"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="0">
-      <formula>$F2="Blocked"</formula>
+      <formula>$G2="Blocked"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="0">
-      <formula>$F2="Done"</formula>
+      <formula>$G2="Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="D2:D25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Nayab,Lumia,Izza,Laiba,Reesha,Hurema,Team,Unassigned"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not started,In progress,Blocked,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1529,7 +1711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1537,120 +1719,132 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Week of Mon 28 Sep 2026 — deadline for the compiled dataset: Sat 03 Oct</t>
         </is>
       </c>
-      <c r="B1" s="3" t="n"/>
+      <c r="B1" s="4" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr"/>
-      <c r="B2" s="3" t="n"/>
+      <c r="A2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Status values</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Not started, In progress, Blocked, Done</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Modules</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Re-annotation, Data augmentation, Transfer evaluation, Span selection, Model tuning, Entrepreneurial data, Specificity set</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Row colour</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>amber = in progress, red = blocked, green = done</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr"/>
-      <c r="B5" s="3" t="n"/>
-    </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr"/>
+      <c r="B6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Standing rules</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Augmentation is TRAIN ONLY; never val or test.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Augmented rows stay in their source row's split, or it is leakage.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Form/interview responses are EVALUATION ONLY — never prompts, never training.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>The test set is never balanced; it stays at its natural distribution.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Thresholds are tuned on val. Test is read once, at the end.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>The challenge set is evaluation only and is frozen once verified.</t>
         </is>

</xml_diff>